<commit_message>
Prepare manuscript package and analysis outputs for GitHub
</commit_message>
<xml_diff>
--- a/manuscript_package/tables/table01_dataset_grouped_structure.xlsx
+++ b/manuscript_package/tables/table01_dataset_grouped_structure.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +25,21 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E8FB"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +54,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -411,184 +425,635 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>metric</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>value</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Statistic</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Unit/Note</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>n_rows</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>1009</v>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Dataset scope</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Observations</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>1009</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>rows</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>n_real_features</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>25</v>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Dataset scope</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Real predictors</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>variables</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>n_studies</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>23</v>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Dataset scope</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>aut_id</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>n_experiments</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>149</v>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Dataset scope</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Experiments</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>149</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>exp_id</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>median_rows_per_study</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>38</v>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Grouped structure</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Median rows per study</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>rows</t>
+        </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>max_rows_per_study</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>180</v>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Grouped structure</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Maximum rows per study</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>180</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>rows</t>
+        </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>median_rows_per_experiment</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>6</v>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Grouped structure</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Median rows per experiment</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>rows</t>
+        </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>max_rows_per_experiment</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>10</v>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Grouped structure</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Maximum rows per experiment</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>rows</t>
+        </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>median_qe</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>0.10325</v>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Target distribution</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Median qe</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>0.103</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>mg g^-1</t>
+        </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>p95_qe</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>5.051816607199997</v>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Target distribution</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>IQR qe</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>0.032-0.454</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>mg g^-1</t>
+        </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>max_qe</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>17.77876</v>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Target distribution</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>95th percentile qe</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>5.052</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>mg g^-1</t>
+        </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>missing_fraction_ph</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>0.533201189296333</v>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Target distribution</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Maximum qe</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>17.779</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>mg g^-1</t>
+        </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>missing_fraction_sa</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>0.379583746283449</v>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Reporting completeness</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Missing pH</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>53.3%</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>of rows</t>
+        </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>rows_metal_cd</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>535</v>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Reporting completeness</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Missing surface area</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>38.0%</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>of rows</t>
+        </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>rows_metal_cr</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>308</v>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Reporting completeness</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Missing temperature</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>10.3%</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>of rows</t>
+        </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>rows_metal_hg</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>166</v>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Reporting completeness</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Missing agitation speed</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>5.4%</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>of rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Metal composition</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Cd(II)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>535 (53.0%)</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>rows (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Metal composition</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Cr(VI)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>308 (30.5%)</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>rows (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Metal composition</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Hg(II)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>166 (16.5%)</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>rows (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Polymer composition</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>154 (15.3%)</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>rows (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Polymer composition</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>PP</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>60 (5.9%)</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>rows (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Polymer composition</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>382 (37.9%)</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>rows (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Polymer composition</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>58 (5.7%)</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>rows (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Polymer composition</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>PET</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>110 (10.9%)</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>rows (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Polymer composition</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>126 (12.5%)</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>rows (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Polymer composition</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>PLA</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>54 (5.4%)</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>rows (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Polymer composition</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>65 (6.4%)</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>rows (%)</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>